<commit_message>
Remove survey from Moodle 5 tool list
</commit_message>
<xml_diff>
--- a/Datenbank_ToolGuide.xlsx
+++ b/Datenbank_ToolGuide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/moskaliuk/Documents/Code/moodletoolguide/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0845BD7C-434A-0247-9626-AECE75B635FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC01B4C-4373-9648-83FD-66E0FEE8F2D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Bloom Taxonomie" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$A$1:$J$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$A$1:$J$96</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1577" uniqueCount="273">
   <si>
     <t>Aktivität</t>
   </si>
@@ -347,28 +347,7 @@
     <t>Ja. Inhalte können bewertet werden. Datenbank ist flexibel einsetzbar.</t>
   </si>
   <si>
-    <t>Umfrage</t>
-  </si>
-  <si>
-    <t>Befragung mit vordefinierten Fragen</t>
-  </si>
-  <si>
-    <t>Einfach. Wähle aus 3 Typen, um Einstellungen und Lernerfahrungen zu erfragen.</t>
-  </si>
-  <si>
-    <t>https://docs.moodle.org/501/de/Umfrage</t>
-  </si>
-  <si>
-    <t>Vorlage wählen, fertig.</t>
-  </si>
-  <si>
-    <t>Keine Pflege – Auswertung am Ende.</t>
-  </si>
-  <si>
     <t>Nein. Ist eine rein individuelle Aktivität von Teilnehmenden.</t>
-  </si>
-  <si>
-    <t>Hilft Teilnehmenden Lernprozess zu reflektieren.</t>
   </si>
   <si>
     <t>Feedback</t>
@@ -870,7 +849,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -923,14 +902,6 @@
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1013,7 +984,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1041,13 +1012,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1352,7 +1316,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R112"/>
+  <dimension ref="A1:R111"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -3338,96 +3302,96 @@
       <c r="R41" s="5"/>
     </row>
     <row r="42" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B42" s="11" t="s">
+      <c r="A42" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="B42" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D42" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="E42" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="F42" s="11" t="s">
+      <c r="C42" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="I42" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="J42" s="6"/>
+      <c r="K42" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="L42" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="M42" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="G42" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="H42" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="I42" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="J42" s="11"/>
-      <c r="K42" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="L42" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="M42" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="N42" s="12" t="s">
+      <c r="N42" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="O42" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="P42" s="12"/>
-      <c r="Q42" s="12"/>
-      <c r="R42" s="12"/>
+      <c r="O42" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="P42" s="5"/>
+      <c r="Q42" s="5"/>
+      <c r="R42" s="5"/>
     </row>
     <row r="43" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="6" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B43" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F43" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>119</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="I43" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J43" s="6"/>
       <c r="K43" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="L43" s="5" t="s">
         <v>59</v>
       </c>
       <c r="M43" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="N43" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O43" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="P43" s="5"/>
       <c r="Q43" s="5"/>
@@ -3435,47 +3399,47 @@
     </row>
     <row r="44" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="6" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C44" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F44" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>123</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J44" s="6"/>
       <c r="K44" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="L44" s="5" t="s">
         <v>59</v>
       </c>
       <c r="M44" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="N44" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O44" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="P44" s="5"/>
       <c r="Q44" s="5"/>
@@ -3483,47 +3447,47 @@
     </row>
     <row r="45" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="6" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="I45" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J45" s="6"/>
       <c r="K45" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="L45" s="5" t="s">
         <v>59</v>
       </c>
       <c r="M45" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="N45" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O45" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="P45" s="5"/>
       <c r="Q45" s="5"/>
@@ -3531,47 +3495,47 @@
     </row>
     <row r="46" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="6" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E46" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="F46" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="F46" s="6" t="s">
+      <c r="G46" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="H46" s="6" t="s">
         <v>113</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>120</v>
       </c>
       <c r="I46" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J46" s="6"/>
       <c r="K46" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>59</v>
       </c>
       <c r="M46" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="N46" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O46" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="P46" s="5"/>
       <c r="Q46" s="5"/>
@@ -3579,47 +3543,47 @@
     </row>
     <row r="47" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>118</v>
+        <v>19</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="G47" s="10" t="s">
-        <v>45</v>
+        <v>122</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="I47" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J47" s="6"/>
       <c r="K47" s="5" t="s">
-        <v>118</v>
+        <v>19</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="M47" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="N47" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O47" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="P47" s="5"/>
       <c r="Q47" s="5"/>
@@ -3627,28 +3591,28 @@
     </row>
     <row r="48" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="6" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>30</v>
+        <v>126</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="I48" s="8" t="s">
         <v>23</v>
@@ -3661,13 +3625,13 @@
         <v>24</v>
       </c>
       <c r="M48" s="5" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="N48" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O48" s="5" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="P48" s="5"/>
       <c r="Q48" s="5"/>
@@ -3675,28 +3639,28 @@
     </row>
     <row r="49" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="6" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E49" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="G49" s="7" t="s">
-        <v>21</v>
+        <v>127</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="I49" s="8" t="s">
         <v>23</v>
@@ -3709,13 +3673,13 @@
         <v>24</v>
       </c>
       <c r="M49" s="5" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="N49" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O49" s="5" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="P49" s="5"/>
       <c r="Q49" s="5"/>
@@ -3723,28 +3687,28 @@
     </row>
     <row r="50" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="6" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="I50" s="8" t="s">
         <v>23</v>
@@ -3757,13 +3721,13 @@
         <v>24</v>
       </c>
       <c r="M50" s="5" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="N50" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O50" s="5" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="P50" s="5"/>
       <c r="Q50" s="5"/>
@@ -3771,28 +3735,28 @@
     </row>
     <row r="51" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="6" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E51" s="6" t="s">
         <v>19</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>30</v>
+        <v>129</v>
+      </c>
+      <c r="G51" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="I51" s="8" t="s">
         <v>23</v>
@@ -3805,13 +3769,13 @@
         <v>24</v>
       </c>
       <c r="M51" s="5" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="N51" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O51" s="5" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="P51" s="5"/>
       <c r="Q51" s="5"/>
@@ -3819,47 +3783,47 @@
     </row>
     <row r="52" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="6" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="G52" s="10" t="s">
-        <v>45</v>
+        <v>133</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="I52" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J52" s="6"/>
       <c r="K52" s="5" t="s">
-        <v>19</v>
+        <v>89</v>
       </c>
       <c r="L52" s="5" t="s">
-        <v>24</v>
+        <v>103</v>
       </c>
       <c r="M52" s="5" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="N52" s="5" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="O52" s="5" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="P52" s="5"/>
       <c r="Q52" s="5"/>
@@ -3867,28 +3831,28 @@
     </row>
     <row r="53" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="6" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="G53" s="9" t="s">
-        <v>30</v>
+        <v>137</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="I53" s="8" t="s">
         <v>23</v>
@@ -3901,13 +3865,13 @@
         <v>103</v>
       </c>
       <c r="M53" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="N53" s="5" t="s">
         <v>59</v>
       </c>
       <c r="O53" s="5" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="P53" s="5"/>
       <c r="Q53" s="5"/>
@@ -3915,28 +3879,28 @@
     </row>
     <row r="54" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="6" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="G54" s="7" t="s">
-        <v>21</v>
+        <v>127</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="I54" s="8" t="s">
         <v>23</v>
@@ -3949,13 +3913,13 @@
         <v>103</v>
       </c>
       <c r="M54" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="N54" s="5" t="s">
         <v>59</v>
       </c>
       <c r="O54" s="5" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="P54" s="5"/>
       <c r="Q54" s="5"/>
@@ -3963,28 +3927,28 @@
     </row>
     <row r="55" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="6" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E55" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="I55" s="8" t="s">
         <v>23</v>
@@ -3997,13 +3961,13 @@
         <v>103</v>
       </c>
       <c r="M55" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="N55" s="5" t="s">
         <v>59</v>
       </c>
       <c r="O55" s="5" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="P55" s="5"/>
       <c r="Q55" s="5"/>
@@ -4011,28 +3975,28 @@
     </row>
     <row r="56" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="6" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="G56" s="9" t="s">
-        <v>30</v>
+        <v>139</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="I56" s="8" t="s">
         <v>23</v>
@@ -4045,13 +4009,13 @@
         <v>103</v>
       </c>
       <c r="M56" s="5" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="N56" s="5" t="s">
         <v>59</v>
       </c>
       <c r="O56" s="5" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="P56" s="5"/>
       <c r="Q56" s="5"/>
@@ -4059,28 +4023,28 @@
     </row>
     <row r="57" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="6" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G57" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I57" s="8" t="s">
         <v>23</v>
@@ -4093,13 +4057,13 @@
         <v>103</v>
       </c>
       <c r="M57" s="5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="N57" s="5" t="s">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="O57" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="P57" s="5"/>
       <c r="Q57" s="5"/>
@@ -4107,28 +4071,28 @@
     </row>
     <row r="58" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="G58" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="I58" s="8" t="s">
         <v>23</v>
@@ -4141,13 +4105,13 @@
         <v>103</v>
       </c>
       <c r="M58" s="5" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="N58" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O58" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="P58" s="5"/>
       <c r="Q58" s="5"/>
@@ -4155,28 +4119,28 @@
     </row>
     <row r="59" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="G59" s="7" t="s">
-        <v>21</v>
+        <v>148</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="I59" s="8" t="s">
         <v>23</v>
@@ -4189,13 +4153,13 @@
         <v>103</v>
       </c>
       <c r="M59" s="5" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="N59" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O59" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="P59" s="5"/>
       <c r="Q59" s="5"/>
@@ -4203,28 +4167,28 @@
     </row>
     <row r="60" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="G60" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="I60" s="8" t="s">
         <v>23</v>
@@ -4237,13 +4201,13 @@
         <v>103</v>
       </c>
       <c r="M60" s="5" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="N60" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O60" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="P60" s="5"/>
       <c r="Q60" s="5"/>
@@ -4251,28 +4215,28 @@
     </row>
     <row r="61" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="6" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E61" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="G61" s="9" t="s">
-        <v>30</v>
+        <v>149</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="I61" s="8" t="s">
         <v>23</v>
@@ -4285,13 +4249,13 @@
         <v>103</v>
       </c>
       <c r="M61" s="5" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="N61" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O61" s="5" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="P61" s="5"/>
       <c r="Q61" s="5"/>
@@ -4299,47 +4263,47 @@
     </row>
     <row r="62" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="6" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="G62" s="7" t="s">
-        <v>21</v>
+        <v>153</v>
+      </c>
+      <c r="G62" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="I62" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J62" s="6"/>
       <c r="K62" s="5" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="L62" s="5" t="s">
-        <v>103</v>
+        <v>24</v>
       </c>
       <c r="M62" s="5" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="N62" s="5" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="O62" s="5" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="P62" s="5"/>
       <c r="Q62" s="5"/>
@@ -4347,28 +4311,28 @@
     </row>
     <row r="63" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E63" s="6" t="s">
         <v>76</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>30</v>
+        <v>157</v>
+      </c>
+      <c r="G63" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="I63" s="8" t="s">
         <v>23</v>
@@ -4381,13 +4345,13 @@
         <v>24</v>
       </c>
       <c r="M63" s="5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="N63" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O63" s="5" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="P63" s="5"/>
       <c r="Q63" s="5"/>
@@ -4395,28 +4359,28 @@
     </row>
     <row r="64" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>76</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="G64" s="7" t="s">
-        <v>21</v>
+        <v>158</v>
+      </c>
+      <c r="G64" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="I64" s="8" t="s">
         <v>23</v>
@@ -4429,13 +4393,13 @@
         <v>24</v>
       </c>
       <c r="M64" s="5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="N64" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O64" s="5" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="P64" s="5"/>
       <c r="Q64" s="5"/>
@@ -4443,28 +4407,28 @@
     </row>
     <row r="65" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>76</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="G65" s="9" t="s">
-        <v>30</v>
+        <v>159</v>
+      </c>
+      <c r="G65" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="I65" s="8" t="s">
         <v>23</v>
@@ -4477,13 +4441,13 @@
         <v>24</v>
       </c>
       <c r="M65" s="5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="N65" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O65" s="5" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="P65" s="5"/>
       <c r="Q65" s="5"/>
@@ -4491,28 +4455,28 @@
     </row>
     <row r="66" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>76</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="G66" s="10" t="s">
-        <v>45</v>
+        <v>160</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="I66" s="8" t="s">
         <v>23</v>
@@ -4525,13 +4489,13 @@
         <v>24</v>
       </c>
       <c r="M66" s="5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="N66" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O66" s="5" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="P66" s="5"/>
       <c r="Q66" s="5"/>
@@ -4539,47 +4503,47 @@
     </row>
     <row r="67" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="6" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="G67" s="7" t="s">
-        <v>21</v>
+        <v>164</v>
+      </c>
+      <c r="G67" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="I67" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J67" s="6"/>
       <c r="K67" s="5" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
       <c r="L67" s="5" t="s">
-        <v>24</v>
+        <v>103</v>
       </c>
       <c r="M67" s="5" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="N67" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O67" s="5" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="P67" s="5"/>
       <c r="Q67" s="5"/>
@@ -4587,28 +4551,28 @@
     </row>
     <row r="68" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="6" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="G68" s="9" t="s">
-        <v>30</v>
+        <v>168</v>
+      </c>
+      <c r="G68" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="I68" s="8" t="s">
         <v>23</v>
@@ -4621,13 +4585,13 @@
         <v>103</v>
       </c>
       <c r="M68" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="N68" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O68" s="5" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="P68" s="5"/>
       <c r="Q68" s="5"/>
@@ -4635,28 +4599,28 @@
     </row>
     <row r="69" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="6" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E69" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="G69" s="7" t="s">
-        <v>21</v>
+        <v>169</v>
+      </c>
+      <c r="G69" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="I69" s="8" t="s">
         <v>23</v>
@@ -4669,13 +4633,13 @@
         <v>103</v>
       </c>
       <c r="M69" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="N69" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O69" s="5" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="P69" s="5"/>
       <c r="Q69" s="5"/>
@@ -4683,28 +4647,28 @@
     </row>
     <row r="70" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="6" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="G70" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="I70" s="8" t="s">
         <v>23</v>
@@ -4717,13 +4681,13 @@
         <v>103</v>
       </c>
       <c r="M70" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="N70" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O70" s="5" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="P70" s="5"/>
       <c r="Q70" s="5"/>
@@ -4731,28 +4695,28 @@
     </row>
     <row r="71" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="6" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E71" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G71" s="9" t="s">
-        <v>30</v>
+        <v>160</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="I71" s="8" t="s">
         <v>23</v>
@@ -4765,13 +4729,13 @@
         <v>103</v>
       </c>
       <c r="M71" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="N71" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O71" s="5" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="P71" s="5"/>
       <c r="Q71" s="5"/>
@@ -4779,47 +4743,47 @@
     </row>
     <row r="72" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="G72" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="I72" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J72" s="6"/>
       <c r="K72" s="5" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="L72" s="5" t="s">
         <v>103</v>
       </c>
       <c r="M72" s="5" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="N72" s="5" t="s">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="O72" s="5" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="P72" s="5"/>
       <c r="Q72" s="5"/>
@@ -4827,28 +4791,28 @@
     </row>
     <row r="73" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="6" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="G73" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="I73" s="8" t="s">
         <v>23</v>
@@ -4861,13 +4825,13 @@
         <v>103</v>
       </c>
       <c r="M73" s="5" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="N73" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O73" s="5" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="P73" s="5"/>
       <c r="Q73" s="5"/>
@@ -4875,28 +4839,28 @@
     </row>
     <row r="74" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="6" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="G74" s="7" t="s">
-        <v>21</v>
+        <v>148</v>
+      </c>
+      <c r="G74" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="I74" s="8" t="s">
         <v>23</v>
@@ -4909,13 +4873,13 @@
         <v>103</v>
       </c>
       <c r="M74" s="5" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="N74" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O74" s="5" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="P74" s="5"/>
       <c r="Q74" s="5"/>
@@ -4923,28 +4887,28 @@
     </row>
     <row r="75" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="6" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E75" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="G75" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="I75" s="8" t="s">
         <v>23</v>
@@ -4957,13 +4921,13 @@
         <v>103</v>
       </c>
       <c r="M75" s="5" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="N75" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O75" s="5" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="P75" s="5"/>
       <c r="Q75" s="5"/>
@@ -4971,28 +4935,28 @@
     </row>
     <row r="76" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="6" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="G76" s="9" t="s">
-        <v>30</v>
+        <v>149</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="I76" s="8" t="s">
         <v>23</v>
@@ -5005,13 +4969,13 @@
         <v>103</v>
       </c>
       <c r="M76" s="5" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="N76" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O76" s="5" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="P76" s="5"/>
       <c r="Q76" s="5"/>
@@ -5019,47 +4983,47 @@
     </row>
     <row r="77" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>156</v>
+        <v>182</v>
       </c>
       <c r="G77" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I77" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J77" s="6"/>
       <c r="K77" s="5" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="L77" s="5" t="s">
-        <v>103</v>
+        <v>24</v>
       </c>
       <c r="M77" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="N77" s="5" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="O77" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="P77" s="5"/>
       <c r="Q77" s="5"/>
@@ -5067,28 +5031,28 @@
     </row>
     <row r="78" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="6" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F78" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="G78" s="7" t="s">
-        <v>21</v>
+        <v>186</v>
+      </c>
+      <c r="G78" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="I78" s="8" t="s">
         <v>23</v>
@@ -5101,13 +5065,13 @@
         <v>24</v>
       </c>
       <c r="M78" s="5" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="N78" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O78" s="5" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="P78" s="5"/>
       <c r="Q78" s="5"/>
@@ -5115,28 +5079,28 @@
     </row>
     <row r="79" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="6" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E79" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="G79" s="10" t="s">
-        <v>45</v>
+        <v>187</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="I79" s="8" t="s">
         <v>23</v>
@@ -5149,13 +5113,13 @@
         <v>24</v>
       </c>
       <c r="M79" s="5" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="N79" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O79" s="5" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="P79" s="5"/>
       <c r="Q79" s="5"/>
@@ -5163,28 +5127,28 @@
     </row>
     <row r="80" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="6" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="G80" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="I80" s="8" t="s">
         <v>23</v>
@@ -5197,13 +5161,13 @@
         <v>24</v>
       </c>
       <c r="M80" s="5" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="N80" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O80" s="5" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="P80" s="5"/>
       <c r="Q80" s="5"/>
@@ -5211,28 +5175,28 @@
     </row>
     <row r="81" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="6" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C81" s="6" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="D81" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E81" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F81" s="6" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="G81" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H81" s="6" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="I81" s="8" t="s">
         <v>23</v>
@@ -5245,13 +5209,13 @@
         <v>24</v>
       </c>
       <c r="M81" s="5" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="N81" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O81" s="5" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="P81" s="5"/>
       <c r="Q81" s="5"/>
@@ -5259,47 +5223,47 @@
     </row>
     <row r="82" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="6" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D82" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="F82" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="G82" s="7" t="s">
-        <v>21</v>
+        <v>193</v>
+      </c>
+      <c r="G82" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="I82" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J82" s="6"/>
       <c r="K82" s="5" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="L82" s="5" t="s">
-        <v>24</v>
+        <v>103</v>
       </c>
       <c r="M82" s="5" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="N82" s="5" t="s">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="O82" s="5" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="P82" s="5"/>
       <c r="Q82" s="5"/>
@@ -5307,28 +5271,28 @@
     </row>
     <row r="83" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="6" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="D83" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E83" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F83" s="6" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="G83" s="10" t="s">
         <v>45</v>
       </c>
       <c r="H83" s="6" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="I83" s="8" t="s">
         <v>23</v>
@@ -5341,13 +5305,13 @@
         <v>103</v>
       </c>
       <c r="M83" s="5" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="N83" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O83" s="5" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="P83" s="5"/>
       <c r="Q83" s="5"/>
@@ -5355,28 +5319,28 @@
     </row>
     <row r="84" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="6" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F84" s="6" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="G84" s="10" t="s">
         <v>45</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="I84" s="8" t="s">
         <v>23</v>
@@ -5389,13 +5353,13 @@
         <v>103</v>
       </c>
       <c r="M84" s="5" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="N84" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O84" s="5" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="P84" s="5"/>
       <c r="Q84" s="5"/>
@@ -5403,28 +5367,28 @@
     </row>
     <row r="85" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="6" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E85" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F85" s="6" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G85" s="10" t="s">
         <v>45</v>
       </c>
       <c r="H85" s="6" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="I85" s="8" t="s">
         <v>23</v>
@@ -5437,13 +5401,13 @@
         <v>103</v>
       </c>
       <c r="M85" s="5" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="N85" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O85" s="5" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="P85" s="5"/>
       <c r="Q85" s="5"/>
@@ -5451,28 +5415,28 @@
     </row>
     <row r="86" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="6" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="D86" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E86" s="6" t="s">
         <v>89</v>
       </c>
       <c r="F86" s="6" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G86" s="10" t="s">
         <v>45</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="I86" s="8" t="s">
         <v>23</v>
@@ -5485,13 +5449,13 @@
         <v>103</v>
       </c>
       <c r="M86" s="5" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="N86" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O86" s="5" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="P86" s="5"/>
       <c r="Q86" s="5"/>
@@ -5499,47 +5463,47 @@
     </row>
     <row r="87" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="6" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="F87" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="G87" s="10" t="s">
-        <v>45</v>
+        <v>202</v>
+      </c>
+      <c r="G87" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H87" s="6" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I87" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J87" s="6"/>
       <c r="K87" s="5" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="L87" s="5" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="M87" s="5" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="N87" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O87" s="5" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="P87" s="5"/>
       <c r="Q87" s="5"/>
@@ -5547,28 +5511,28 @@
     </row>
     <row r="88" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="6" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C88" s="6" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D88" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F88" s="6" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="G88" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="I88" s="8" t="s">
         <v>23</v>
@@ -5581,13 +5545,13 @@
         <v>59</v>
       </c>
       <c r="M88" s="5" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="N88" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O88" s="5" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="P88" s="5"/>
       <c r="Q88" s="5"/>
@@ -5595,28 +5559,28 @@
     </row>
     <row r="89" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="6" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C89" s="6" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D89" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E89" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F89" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="G89" s="7" t="s">
-        <v>21</v>
+        <v>207</v>
+      </c>
+      <c r="G89" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="H89" s="6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="I89" s="8" t="s">
         <v>23</v>
@@ -5629,13 +5593,13 @@
         <v>59</v>
       </c>
       <c r="M89" s="5" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="N89" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O89" s="5" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="P89" s="5"/>
       <c r="Q89" s="5"/>
@@ -5643,28 +5607,28 @@
     </row>
     <row r="90" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="6" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D90" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E90" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F90" s="6" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="G90" s="9" t="s">
         <v>30</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="I90" s="8" t="s">
         <v>23</v>
@@ -5677,13 +5641,13 @@
         <v>59</v>
       </c>
       <c r="M90" s="5" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="N90" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O90" s="5" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="P90" s="5"/>
       <c r="Q90" s="5"/>
@@ -5691,28 +5655,28 @@
     </row>
     <row r="91" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="6" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D91" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E91" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F91" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="G91" s="9" t="s">
-        <v>30</v>
+        <v>209</v>
+      </c>
+      <c r="G91" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H91" s="6" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="I91" s="8" t="s">
         <v>23</v>
@@ -5725,13 +5689,13 @@
         <v>59</v>
       </c>
       <c r="M91" s="5" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="N91" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O91" s="5" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="P91" s="5"/>
       <c r="Q91" s="5"/>
@@ -5739,28 +5703,28 @@
     </row>
     <row r="92" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="6" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="D92" s="6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E92" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="G92" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="I92" s="8" t="s">
         <v>23</v>
@@ -5770,16 +5734,16 @@
         <v>100</v>
       </c>
       <c r="L92" s="5" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="M92" s="5" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="N92" s="5" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="O92" s="5" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="P92" s="5"/>
       <c r="Q92" s="5"/>
@@ -5787,28 +5751,28 @@
     </row>
     <row r="93" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="6" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D93" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E93" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F93" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="G93" s="7" t="s">
-        <v>21</v>
+        <v>217</v>
+      </c>
+      <c r="G93" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="H93" s="6" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="I93" s="8" t="s">
         <v>23</v>
@@ -5821,13 +5785,13 @@
         <v>24</v>
       </c>
       <c r="M93" s="5" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="N93" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O93" s="5" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="P93" s="5"/>
       <c r="Q93" s="5"/>
@@ -5835,28 +5799,28 @@
     </row>
     <row r="94" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="6" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C94" s="6" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F94" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="G94" s="10" t="s">
-        <v>45</v>
+        <v>218</v>
+      </c>
+      <c r="G94" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="I94" s="8" t="s">
         <v>23</v>
@@ -5869,13 +5833,13 @@
         <v>24</v>
       </c>
       <c r="M94" s="5" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="N94" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O94" s="5" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="P94" s="5"/>
       <c r="Q94" s="5"/>
@@ -5883,28 +5847,28 @@
     </row>
     <row r="95" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="6" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D95" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E95" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F95" s="6" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="G95" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H95" s="6" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="I95" s="8" t="s">
         <v>23</v>
@@ -5917,13 +5881,13 @@
         <v>24</v>
       </c>
       <c r="M95" s="5" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="N95" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O95" s="5" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="P95" s="5"/>
       <c r="Q95" s="5"/>
@@ -5931,28 +5895,28 @@
     </row>
     <row r="96" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="6" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="D96" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E96" s="6" t="s">
         <v>100</v>
       </c>
       <c r="F96" s="6" t="s">
-        <v>226</v>
+        <v>209</v>
       </c>
       <c r="G96" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="I96" s="8" t="s">
         <v>23</v>
@@ -5965,61 +5929,61 @@
         <v>24</v>
       </c>
       <c r="M96" s="5" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="N96" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O96" s="5" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="P96" s="5"/>
       <c r="Q96" s="5"/>
       <c r="R96" s="5"/>
     </row>
     <row r="97" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="B97" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="C97" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="D97" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E97" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="F97" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="G97" s="7" t="s">
+      <c r="A97" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C97" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="D97" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F97" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="G97" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H97" s="6" t="s">
-        <v>221</v>
+      <c r="H97" s="5" t="s">
+        <v>224</v>
       </c>
       <c r="I97" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="J97" s="6"/>
+      <c r="J97" s="5"/>
       <c r="K97" s="5" t="s">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="L97" s="5" t="s">
         <v>24</v>
       </c>
       <c r="M97" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="N97" s="5" t="s">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="O97" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="P97" s="5"/>
       <c r="Q97" s="5"/>
@@ -6027,47 +5991,47 @@
     </row>
     <row r="98" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="B98" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C98" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="D98" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E98" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F98" s="5" t="s">
         <v>227</v>
       </c>
-      <c r="B98" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="C98" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="D98" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="F98" s="5" t="s">
-        <v>230</v>
-      </c>
       <c r="G98" s="5" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="H98" s="5" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="I98" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J98" s="5"/>
       <c r="K98" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="L98" s="5" t="s">
         <v>24</v>
       </c>
       <c r="M98" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="N98" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O98" s="5" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="P98" s="5"/>
       <c r="Q98" s="5"/>
@@ -6075,47 +6039,47 @@
     </row>
     <row r="99" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="5" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B99" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C99" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="D99" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E99" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F99" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="C99" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="D99" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="E99" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="F99" s="5" t="s">
-        <v>234</v>
-      </c>
       <c r="G99" s="5" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="H99" s="5" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="I99" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J99" s="5"/>
       <c r="K99" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="L99" s="5" t="s">
         <v>24</v>
       </c>
       <c r="M99" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="N99" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O99" s="5" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="P99" s="5"/>
       <c r="Q99" s="5"/>
@@ -6123,47 +6087,47 @@
     </row>
     <row r="100" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="5" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B100" s="5" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="C100" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="D100" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E100" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="F100" s="5" t="s">
         <v>229</v>
-      </c>
-      <c r="D100" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="F100" s="5" t="s">
-        <v>235</v>
       </c>
       <c r="G100" s="5" t="s">
         <v>21</v>
       </c>
       <c r="H100" s="5" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="I100" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J100" s="5"/>
       <c r="K100" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="L100" s="5" t="s">
         <v>24</v>
       </c>
       <c r="M100" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="N100" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O100" s="5" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="P100" s="5"/>
       <c r="Q100" s="5"/>
@@ -6171,47 +6135,47 @@
     </row>
     <row r="101" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="5" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B101" s="5" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="C101" s="5" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="D101" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F101" s="5" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="G101" s="5" t="s">
         <v>21</v>
       </c>
       <c r="H101" s="5" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="I101" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J101" s="5"/>
       <c r="K101" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="L101" s="5" t="s">
         <v>24</v>
       </c>
       <c r="M101" s="5" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="N101" s="5" t="s">
         <v>26</v>
       </c>
       <c r="O101" s="5" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="P101" s="5"/>
       <c r="Q101" s="5"/>
@@ -6219,47 +6183,47 @@
     </row>
     <row r="102" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="5" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="B102" s="5" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D102" s="5" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>118</v>
+        <v>19</v>
       </c>
       <c r="F102" s="5" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="G102" s="5" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="H102" s="5" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="I102" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J102" s="5"/>
       <c r="K102" s="5" t="s">
-        <v>118</v>
+        <v>19</v>
       </c>
       <c r="L102" s="5" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="M102" s="5" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="N102" s="5" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="O102" s="5" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="P102" s="5"/>
       <c r="Q102" s="5"/>
@@ -6267,28 +6231,28 @@
     </row>
     <row r="103" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="5" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B103" s="5" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C103" s="5" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D103" s="5" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E103" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F103" s="5" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G103" s="5" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="H103" s="5" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="I103" s="8" t="s">
         <v>23</v>
@@ -6301,13 +6265,13 @@
         <v>59</v>
       </c>
       <c r="M103" s="5" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="N103" s="5" t="s">
         <v>59</v>
       </c>
       <c r="O103" s="5" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="P103" s="5"/>
       <c r="Q103" s="5"/>
@@ -6315,28 +6279,28 @@
     </row>
     <row r="104" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="5" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B104" s="5" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C104" s="5" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D104" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E104" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F104" s="5" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="G104" s="5" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H104" s="5" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="I104" s="8" t="s">
         <v>23</v>
@@ -6349,13 +6313,13 @@
         <v>59</v>
       </c>
       <c r="M104" s="5" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="N104" s="5" t="s">
         <v>59</v>
       </c>
       <c r="O104" s="5" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="P104" s="5"/>
       <c r="Q104" s="5"/>
@@ -6363,28 +6327,28 @@
     </row>
     <row r="105" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="5" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B105" s="5" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C105" s="5" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D105" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E105" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F105" s="5" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="G105" s="5" t="s">
         <v>30</v>
       </c>
       <c r="H105" s="5" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="I105" s="8" t="s">
         <v>23</v>
@@ -6397,13 +6361,13 @@
         <v>59</v>
       </c>
       <c r="M105" s="5" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="N105" s="5" t="s">
         <v>59</v>
       </c>
       <c r="O105" s="5" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="P105" s="5"/>
       <c r="Q105" s="5"/>
@@ -6411,28 +6375,28 @@
     </row>
     <row r="106" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="5" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B106" s="5" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="C106" s="5" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="D106" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E106" s="5" t="s">
         <v>19</v>
       </c>
       <c r="F106" s="5" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="G106" s="5" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="H106" s="5" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="I106" s="8" t="s">
         <v>23</v>
@@ -6445,13 +6409,13 @@
         <v>59</v>
       </c>
       <c r="M106" s="5" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="N106" s="5" t="s">
         <v>59</v>
       </c>
       <c r="O106" s="5" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="P106" s="5"/>
       <c r="Q106" s="5"/>
@@ -6459,47 +6423,47 @@
     </row>
     <row r="107" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="5" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="B107" s="5" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="C107" s="5" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D107" s="5" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>19</v>
+        <v>100</v>
       </c>
       <c r="F107" s="5" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="G107" s="5" t="s">
         <v>45</v>
       </c>
       <c r="H107" s="5" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="I107" s="8" t="s">
         <v>23</v>
       </c>
       <c r="J107" s="5"/>
       <c r="K107" s="5" t="s">
-        <v>19</v>
+        <v>100</v>
       </c>
       <c r="L107" s="5" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="M107" s="5" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="N107" s="5" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="O107" s="5" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="P107" s="5"/>
       <c r="Q107" s="5"/>
@@ -6507,28 +6471,28 @@
     </row>
     <row r="108" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="5" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="B108" s="5" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C108" s="5" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D108" s="5" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E108" s="5" t="s">
         <v>100</v>
       </c>
       <c r="F108" s="5" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="G108" s="5" t="s">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="H108" s="5" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="I108" s="8" t="s">
         <v>23</v>
@@ -6541,13 +6505,13 @@
         <v>24</v>
       </c>
       <c r="M108" s="5" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="N108" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O108" s="5" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="P108" s="5"/>
       <c r="Q108" s="5"/>
@@ -6555,28 +6519,28 @@
     </row>
     <row r="109" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="5" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="B109" s="5" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C109" s="5" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D109" s="5" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E109" s="5" t="s">
         <v>100</v>
       </c>
       <c r="F109" s="5" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="G109" s="5" t="s">
         <v>21</v>
       </c>
       <c r="H109" s="5" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="I109" s="8" t="s">
         <v>23</v>
@@ -6589,13 +6553,13 @@
         <v>24</v>
       </c>
       <c r="M109" s="5" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="N109" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O109" s="5" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="P109" s="5"/>
       <c r="Q109" s="5"/>
@@ -6603,28 +6567,28 @@
     </row>
     <row r="110" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="5" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="B110" s="5" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C110" s="5" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D110" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E110" s="5" t="s">
         <v>100</v>
       </c>
       <c r="F110" s="5" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="G110" s="5" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="H110" s="5" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="I110" s="8" t="s">
         <v>23</v>
@@ -6637,13 +6601,13 @@
         <v>24</v>
       </c>
       <c r="M110" s="5" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="N110" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O110" s="5" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="P110" s="5"/>
       <c r="Q110" s="5"/>
@@ -6651,28 +6615,28 @@
     </row>
     <row r="111" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="5" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="B111" s="5" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="C111" s="5" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D111" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E111" s="5" t="s">
         <v>100</v>
       </c>
       <c r="F111" s="5" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="G111" s="5" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="H111" s="5" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="I111" s="8" t="s">
         <v>23</v>
@@ -6685,68 +6649,20 @@
         <v>24</v>
       </c>
       <c r="M111" s="5" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="N111" s="5" t="s">
         <v>80</v>
       </c>
       <c r="O111" s="5" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="P111" s="5"/>
       <c r="Q111" s="5"/>
       <c r="R111" s="5"/>
     </row>
-    <row r="112" spans="1:18" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="B112" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="C112" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="D112" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="E112" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="F112" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="G112" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H112" s="5" t="s">
-        <v>253</v>
-      </c>
-      <c r="I112" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="J112" s="5"/>
-      <c r="K112" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="L112" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="M112" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="N112" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="O112" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="P112" s="5"/>
-      <c r="Q112" s="5"/>
-      <c r="R112" s="5"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J97" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:J96" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="I3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
@@ -6788,77 +6704,76 @@
     <hyperlink ref="I39" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
     <hyperlink ref="I40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
     <hyperlink ref="I41" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="I42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="I43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="I44" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="I45" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="I46" r:id="rId45" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="I47" r:id="rId46" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="I48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="I49" r:id="rId48" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="I50" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="I51" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="I52" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="I53" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="I54" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="I55" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="I56" r:id="rId55" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="I57" r:id="rId56" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="I58" r:id="rId57" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="I59" r:id="rId58" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="I60" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="I61" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="I62" r:id="rId61" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="I63" r:id="rId62" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="I64" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="I65" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="I66" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="I67" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="I68" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="I69" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="I70" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="I71" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="I72" r:id="rId71" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="I73" r:id="rId72" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="I74" r:id="rId73" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="I75" r:id="rId74" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="I76" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="I77" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="I78" r:id="rId77" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
-    <hyperlink ref="I79" r:id="rId78" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="I80" r:id="rId79" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
-    <hyperlink ref="I81" r:id="rId80" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="I82" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
-    <hyperlink ref="I83" r:id="rId82" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
-    <hyperlink ref="I84" r:id="rId83" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
-    <hyperlink ref="I85" r:id="rId84" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
-    <hyperlink ref="I86" r:id="rId85" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
-    <hyperlink ref="I87" r:id="rId86" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
-    <hyperlink ref="I88" r:id="rId87" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
-    <hyperlink ref="I89" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
-    <hyperlink ref="I90" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
-    <hyperlink ref="I91" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
-    <hyperlink ref="I92" r:id="rId91" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
-    <hyperlink ref="I93" r:id="rId92" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
-    <hyperlink ref="I94" r:id="rId93" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
-    <hyperlink ref="I95" r:id="rId94" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
-    <hyperlink ref="I96" r:id="rId95" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
-    <hyperlink ref="I97" r:id="rId96" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
-    <hyperlink ref="I98" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
-    <hyperlink ref="I99" r:id="rId98" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
-    <hyperlink ref="I100" r:id="rId99" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
-    <hyperlink ref="I101" r:id="rId100" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
-    <hyperlink ref="I102" r:id="rId101" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
-    <hyperlink ref="I103" r:id="rId102" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
-    <hyperlink ref="I104" r:id="rId103" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
-    <hyperlink ref="I105" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
-    <hyperlink ref="I106" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
-    <hyperlink ref="I107" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
-    <hyperlink ref="I108" r:id="rId107" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
-    <hyperlink ref="I109" r:id="rId108" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
-    <hyperlink ref="I110" r:id="rId109" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
-    <hyperlink ref="I111" r:id="rId110" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
-    <hyperlink ref="I112" r:id="rId111" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
+    <hyperlink ref="I42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="I43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="I44" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="I45" r:id="rId44" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="I46" r:id="rId45" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="I47" r:id="rId46" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="I48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="I49" r:id="rId48" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="I50" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="I51" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="I52" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="I53" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="I54" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="I55" r:id="rId54" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="I56" r:id="rId55" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="I57" r:id="rId56" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="I58" r:id="rId57" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="I59" r:id="rId58" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="I60" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="I61" r:id="rId60" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="I62" r:id="rId61" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="I63" r:id="rId62" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="I64" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="I65" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="I66" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="I67" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="I68" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="I69" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="I70" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="I71" r:id="rId70" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="I72" r:id="rId71" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="I73" r:id="rId72" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="I74" r:id="rId73" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="I75" r:id="rId74" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="I76" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="I77" r:id="rId76" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="I78" r:id="rId77" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="I79" r:id="rId78" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="I80" r:id="rId79" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="I81" r:id="rId80" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="I82" r:id="rId81" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="I83" r:id="rId82" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="I84" r:id="rId83" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="I85" r:id="rId84" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="I86" r:id="rId85" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="I87" r:id="rId86" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="I88" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="I89" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="I90" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="I91" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="I92" r:id="rId91" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="I93" r:id="rId92" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="I94" r:id="rId93" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="I95" r:id="rId94" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="I96" r:id="rId95" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="I97" r:id="rId96" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="I98" r:id="rId97" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="I99" r:id="rId98" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="I100" r:id="rId99" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="I101" r:id="rId100" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="I102" r:id="rId101" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="I103" r:id="rId102" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="I104" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="I105" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="I106" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="I107" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="I108" r:id="rId107" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="I109" r:id="rId108" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="I110" r:id="rId109" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="I111" r:id="rId110" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -6878,16 +6793,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -6895,13 +6810,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -6909,13 +6824,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -6923,13 +6838,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="42" x14ac:dyDescent="0.2">
@@ -6937,13 +6852,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -6954,10 +6869,10 @@
         <v>28</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28" x14ac:dyDescent="0.2">
@@ -6965,13 +6880,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>